<commit_message>
Prepare technical assessment for Midas Health Services
</commit_message>
<xml_diff>
--- a/Documentation/Bug Reporting - WorkForcePro .xlsx
+++ b/Documentation/Bug Reporting - WorkForcePro .xlsx
@@ -188,7 +188,7 @@
 2. View certification expiring in 20 days.</t>
   </si>
   <si>
-    <t>No alert message is shown.</t>
+    <t>No alert message is displayed.</t>
   </si>
   <si>
     <t>Alert message should be displayed.</t>
@@ -233,7 +233,7 @@
   </si>
   <si>
     <t>1. Login as Employee.
-2. View expired certification.</t>
+2. View expired certification</t>
   </si>
   <si>
     <t>Certification is displayed as a normal active certification.</t>

</xml_diff>